<commit_message>
run two items OK
</commit_message>
<xml_diff>
--- a/tests/resources/test_data/TestCases.xlsx
+++ b/tests/resources/test_data/TestCases.xlsx
@@ -60,16 +60,16 @@
     <t xml:space="preserve">Ahoj,babi</t>
   </si>
   <si>
-    <t xml:space="preserve">Ahoj babi</t>
+    <t xml:space="preserve">Ahoj, babi</t>
   </si>
   <si>
     <t xml:space="preserve">Wrong format viz</t>
   </si>
   <si>
-    <t xml:space="preserve">viz.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">viz</t>
+    <t xml:space="preserve">Ahoj,babi,znovu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ahoj, babi, znovu</t>
   </si>
   <si>
     <t xml:space="preserve">default</t>
@@ -313,7 +313,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="1" width="20.76"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="1" width="26.42"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="32.05"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="1" width="11.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="18.49"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="20.76"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="8" style="1" width="11.53"/>
   </cols>
   <sheetData>

</xml_diff>

<commit_message>
clea up, add ${fixes_count} only placeholder
</commit_message>
<xml_diff>
--- a/tests/resources/test_data/TestCases.xlsx
+++ b/tests/resources/test_data/TestCases.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="18">
   <si>
     <t xml:space="preserve">*** Test Cases ***</t>
   </si>
@@ -43,6 +43,9 @@
   </si>
   <si>
     <t xml:space="preserve">${expected}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">${fixes_count}</t>
   </si>
   <si>
     <t xml:space="preserve">Space after comma</t>
@@ -307,7 +310,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="1" width="20.76"/>
@@ -315,7 +318,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="32.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="18.49"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="20.76"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="8" style="1" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="12.84"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="9" style="1" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -340,51 +344,60 @@
       <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="H2" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="H3" s="1" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -411,7 +424,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -438,10 +451,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
make data file dynamic and add csv
</commit_message>
<xml_diff>
--- a/tests/resources/test_data/TestCases.xlsx
+++ b/tests/resources/test_data/TestCases.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="42">
   <si>
     <t xml:space="preserve">*** Test Cases ***</t>
   </si>
@@ -75,7 +75,79 @@
     <t xml:space="preserve">Ahoj, babi, znovu</t>
   </si>
   <si>
-    <t xml:space="preserve">default</t>
+    <t xml:space="preserve">Czech (traditional rules)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bulgarian</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Croatian</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Danish</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dutch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">English (UK)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">English (US)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estonian</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Finnish</t>
+  </si>
+  <si>
+    <t xml:space="preserve">French</t>
+  </si>
+  <si>
+    <t xml:space="preserve">German (Germany)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Greek</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hungarian</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Irish</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Italian</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Latvian</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lithuanian</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maltese</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Polish</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Portuguese</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Romanian</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Slovak</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Slovenian</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spanish</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Swedish</t>
   </si>
 </sst>
 </file>
@@ -401,6 +473,20 @@
       </c>
     </row>
   </sheetData>
+  <dataValidations count="3">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="A1:A1003" type="none">
+      <formula1>0</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="D2:D100" type="list">
+      <formula1>languages!$A$1:$A$26</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="E2:E100" type="list">
+      <formula1>preferences!$A$1:$A$50</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -416,15 +502,140 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1"/>
+  <dimension ref="A1:A26"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="4" width="26.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="3" width="26.42"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
         <v>10</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="3" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="3" t="s">
+        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -453,9 +664,7 @@
       <c r="A1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="4" t="s">
-        <v>17</v>
-      </c>
+      <c r="B1" s="4"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
add files and excel info
</commit_message>
<xml_diff>
--- a/tests/resources/test_data/TestCases.xlsx
+++ b/tests/resources/test_data/TestCases.xlsx
@@ -5,12 +5,13 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="tc" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="languages" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="preferences" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Sheet4" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -22,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="58">
   <si>
     <t xml:space="preserve">*** Test Cases ***</t>
   </si>
@@ -148,6 +149,54 @@
   </si>
   <si>
     <t xml:space="preserve">Swedish</t>
+  </si>
+  <si>
+    <t xml:space="preserve">add test entru není exit </t>
+  </si>
+  <si>
+    <t xml:space="preserve">7 tis. € (Czech, Slovenian)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7 tys. € (Polish)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20 mil. € (many languages)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11 млн. (Bulgarian)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8 mio. (Danish)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">210 miljard = 210 mld. (Dutch)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24 Mio. (German)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">30 τρισ. (Greek)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8 mrd (Hungarian)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12 tūkst. (Lithuanian, Latvian)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20 tn (Swedish)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6 tuh (Estonian)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 tril., 1 mie, 10 mii, 1 milion (Romanian)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2kg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">all languages</t>
   </si>
 </sst>
 </file>
@@ -238,7 +287,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -259,6 +308,14 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -269,6 +326,201 @@
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>528480</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>80280</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="Image 1"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="13993560" cy="3981600"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>679680</xdr:colOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>5040</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Image 2"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId2"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="812880" y="4551840"/>
+          <a:ext cx="4743720" cy="1142640"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>197280</xdr:colOff>
+      <xdr:row>52</xdr:row>
+      <xdr:rowOff>50400</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Image 3"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId3"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="812880" y="5852160"/>
+          <a:ext cx="5886720" cy="5200920"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>59</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>529920</xdr:colOff>
+      <xdr:row>90</xdr:row>
+      <xdr:rowOff>59760</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Image 4"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId4"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="812880" y="12140640"/>
+          <a:ext cx="14807880" cy="5099040"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>92</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>709200</xdr:colOff>
+      <xdr:row>147</xdr:row>
+      <xdr:rowOff>157320</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Image 5"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId5"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="812880" y="17505000"/>
+          <a:ext cx="14174280" cy="9098280"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -382,7 +634,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="1" width="20.76"/>
@@ -451,7 +703,7 @@
         <v>14</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>9</v>
@@ -471,6 +723,63 @@
       <c r="H3" s="1" t="n">
         <v>2</v>
       </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F4" s="0"/>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F5" s="0"/>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F6" s="0"/>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F7" s="0"/>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F8" s="0"/>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F9" s="0"/>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F10" s="0"/>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F11" s="0"/>
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F12" s="0"/>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F13" s="0"/>
+    </row>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F14" s="0"/>
+    </row>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F15" s="0"/>
+    </row>
+    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F16" s="0"/>
+    </row>
+    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F17" s="0"/>
+    </row>
+    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F18" s="0"/>
+    </row>
+    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F19" s="0"/>
+    </row>
+    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F20" s="0"/>
+    </row>
+    <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F21" s="0"/>
+    </row>
+    <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F22" s="0"/>
     </row>
   </sheetData>
   <dataValidations count="3">
@@ -675,4 +984,139 @@
     <oddFooter>&amp;C&amp;"Times New Roman,obyčejné"&amp;12Stránka &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <tabColor rgb="FFFF00FF"/>
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="B27:L57"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="41.13"/>
+  </cols>
+  <sheetData>
+    <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B27" s="0" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="34" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K39" s="5" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="23.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K40" s="5" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="34" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K41" s="5" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="23.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K42" s="5" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="23.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K43" s="5" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="34" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K44" s="5" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="23.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K45" s="5" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="23.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K46" s="5" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="23.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K47" s="5" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="34" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K48" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="23.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K49" s="5" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="23.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K50" s="5" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="44.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K51" s="5" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K52" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="L52" s="6" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K53" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="L53" s="6"/>
+    </row>
+    <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K54" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="L54" s="6"/>
+    </row>
+    <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K55" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="L55" s="6"/>
+    </row>
+    <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K56" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="L56" s="6"/>
+    </row>
+    <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K57" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="L57" s="6"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="L52:L57"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,obyčejné"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,obyčejné"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
2 TEST OK &xxx!!!
</commit_message>
<xml_diff>
--- a/tests/resources/test_data/TestCases.xlsx
+++ b/tests/resources/test_data/TestCases.xlsx
@@ -8,8 +8,8 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="tc_A3" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="tc_final" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="tc_final" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="tc_A3" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="tc" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="languages" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="preferences" sheetId="5" state="visible" r:id="rId7"/>
@@ -17,8 +17,8 @@
     <sheet name="_pattern" sheetId="7" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">tc_A3!$A$1:$G$7</definedName>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">tc_final!$A$1:$G$7</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">tc_A3!$A$1:$G$7</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">tc_final!$A$1:$G$7</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -53,21 +53,10 @@
     <t xml:space="preserve">${fixes_count}</t>
   </si>
   <si>
-    <t xml:space="preserve">45. Correct form of C. a K. in Czech [Czech (academic rules)]</t>
+    <t xml:space="preserve">44. Guns N’ Roses [Czech (academic rules)]</t>
   </si>
   <si>
     <t xml:space="preserve">Czech (academic rules)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C.a k.
-C. a k.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C.&amp;nbsp;a&amp;nbsp;k.
-C.&amp;nbsp;a&amp;nbsp;k.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">44. Guns N’ Roses [Czech (academic rules)]</t>
   </si>
   <si>
     <t xml:space="preserve">Guns’N’Roses
@@ -84,6 +73,17 @@
   </si>
   <si>
     <t xml:space="preserve">Czech (traditional rules)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">45. Correct form of C. a K. in Czech [Czech (academic rules)]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C.a k.
+C. a k.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C.&amp;nbsp;a&amp;nbsp;k.
+C.&amp;nbsp;a&amp;nbsp;k.</t>
   </si>
   <si>
     <t xml:space="preserve">45. Correct form of C. a K. in Czech [Czech (traditional rules)]</t>
@@ -377,7 +377,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -395,11 +395,15 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -653,7 +657,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="58.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
         <v>7</v>
       </c>
@@ -665,57 +669,107 @@
       <c r="E2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="4" t="s">
         <v>10</v>
       </c>
       <c r="G2" s="3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="78.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G4" s="3" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="4"/>
-      <c r="G3" s="3"/>
-    </row>
-    <row r="4" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3"/>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
-    </row>
     <row r="5" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3"/>
+      <c r="A5" s="3" t="s">
+        <v>16</v>
+      </c>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
+      <c r="D5" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3"/>
+      <c r="A6" s="3" t="s">
+        <v>17</v>
+      </c>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3"/>
+      <c r="D6" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3"/>
+      <c r="A7" s="3" t="s">
+        <v>20</v>
+      </c>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
+      <c r="D7" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="3"/>
@@ -9200,7 +9254,7 @@
   <autoFilter ref="A1:G7"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -9249,9 +9303,9 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="58.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -9259,109 +9313,59 @@
         <v>8</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
-      <c r="F2" s="5" t="s">
-        <v>13</v>
+      <c r="F2" s="3" t="s">
+        <v>15</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="78.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
-        <v>14</v>
-      </c>
+    <row r="3" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3"/>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
-      <c r="D3" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G3" s="3" t="n">
-        <v>1</v>
-      </c>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="6"/>
+      <c r="G3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
-        <v>7</v>
-      </c>
+      <c r="A4" s="3"/>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
-      <c r="D4" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="G4" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
     </row>
     <row r="5" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
-        <v>16</v>
-      </c>
+      <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
-      <c r="D5" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="G5" s="3" t="n">
-        <v>2</v>
-      </c>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
     </row>
     <row r="6" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
-        <v>17</v>
-      </c>
+      <c r="A6" s="3"/>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
-      <c r="D6" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="G6" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
     </row>
     <row r="7" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
-        <v>20</v>
-      </c>
+      <c r="A7" s="3"/>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
-      <c r="D7" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="G7" s="3" t="n">
-        <v>3</v>
-      </c>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
     </row>
     <row r="8" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="3"/>
@@ -17846,7 +17850,7 @@
   <autoFilter ref="A1:G7"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -17953,7 +17957,7 @@
         <v>23</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>32</v>
@@ -17976,7 +17980,7 @@
         <v>23</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>36</v>
@@ -18042,7 +18046,7 @@
     </row>
     <row r="2" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18293,75 +18297,75 @@
       </c>
     </row>
     <row r="39" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="K39" s="6" t="s">
+      <c r="K39" s="7" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="K40" s="6" t="s">
+      <c r="K40" s="7" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="K41" s="6" t="s">
+      <c r="K41" s="7" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="K42" s="6" t="s">
+      <c r="K42" s="7" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="K43" s="6" t="s">
+      <c r="K43" s="7" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="K44" s="6" t="s">
+      <c r="K44" s="7" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="K45" s="6" t="s">
+      <c r="K45" s="7" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="K46" s="6" t="s">
+      <c r="K46" s="7" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="K47" s="6" t="s">
+      <c r="K47" s="7" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="K48" s="6" t="s">
+      <c r="K48" s="7" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="K49" s="6" t="s">
+      <c r="K49" s="7" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="K50" s="6" t="s">
+      <c r="K50" s="7" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="K51" s="6" t="s">
+      <c r="K51" s="7" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="K52" s="6" t="s">
+      <c r="K52" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="L52" s="7" t="s">
+      <c r="L52" s="8" t="s">
         <v>79</v>
       </c>
     </row>
@@ -18369,31 +18373,31 @@
       <c r="K53" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="L53" s="7"/>
+      <c r="L53" s="8"/>
     </row>
     <row r="54" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="K54" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="L54" s="7"/>
+      <c r="L54" s="8"/>
     </row>
     <row r="55" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="K55" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="L55" s="7"/>
+      <c r="L55" s="8"/>
     </row>
     <row r="56" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="K56" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="L56" s="7"/>
+      <c r="L56" s="8"/>
     </row>
     <row r="57" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="K57" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="L57" s="7"/>
+      <c r="L57" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
add pcx inactive link 3
</commit_message>
<xml_diff>
--- a/tests/resources/test_data/TestCases.xlsx
+++ b/tests/resources/test_data/TestCases.xlsx
@@ -132,14 +132,14 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="bottom" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
@@ -163,14 +163,14 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="bottom" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
@@ -461,14 +461,14 @@
           <t>Czech (academic rules)</t>
         </is>
       </c>
-      <c r="E2" s="15" t="inlineStr">
+      <c r="E2" s="16" t="inlineStr">
         <is>
           <t>Guns’N’Roses
 Guns n'Roses
 Guns ‘N’ Roses</t>
         </is>
       </c>
-      <c r="F2" s="16" t="inlineStr">
+      <c r="F2" s="17" t="inlineStr">
         <is>
           <t>Guns N’ Roses
 Guns n’Roses
@@ -489,12 +489,11 @@
           <t>2026-05-20T03:10:52.686455</t>
         </is>
       </c>
-      <c r="L2" s="17" t="n"/>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>C:\Users\ocape\IdeaProjects\TypofixAppTest\tests\resources\selenium-element-screenshot-9.png</t>
-        </is>
-      </c>
+      <c r="L2" s="18">
+        <f>HYPERLINK("C:\Users\ocape\IdeaProjects\TypofixAppTest\results\selenium-element-screenshot-9.png", "LINK")</f>
+        <v/>
+      </c>
+      <c r="M2" s="11" t="n"/>
     </row>
     <row r="3" ht="78" customHeight="1" s="12">
       <c r="A3" s="15" t="inlineStr">
@@ -509,14 +508,14 @@
           <t>Czech (traditional rules)</t>
         </is>
       </c>
-      <c r="E3" s="18" t="inlineStr">
+      <c r="E3" s="16" t="inlineStr">
         <is>
           <t>Guns’N’Roses
 Guns n'Roses
 Guns ‘N’ Roses</t>
         </is>
       </c>
-      <c r="F3" s="16" t="inlineStr">
+      <c r="F3" s="17" t="inlineStr">
         <is>
           <t>Guns N’ Roses
 Guns n’Roses
@@ -537,12 +536,11 @@
           <t>2026-05-20T03:11:01.560806</t>
         </is>
       </c>
-      <c r="L3" s="11" t="n"/>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>C:\Users\ocape\IdeaProjects\TypofixAppTest\tests\resources\selenium-element-screenshot-10.png</t>
-        </is>
-      </c>
+      <c r="L3" s="11">
+        <f>HYPERLINK("C:\Users\ocape\IdeaProjects\TypofixAppTest\results\selenium-element-screenshot-10.png", "LINK")</f>
+        <v/>
+      </c>
+      <c r="M3" s="11" t="n"/>
     </row>
     <row r="4" ht="12.75" customHeight="1" s="12">
       <c r="A4" s="15" t="inlineStr">
@@ -557,13 +555,13 @@
           <t>Czech (academic rules)</t>
         </is>
       </c>
-      <c r="E4" s="18" t="inlineStr">
+      <c r="E4" s="16" t="inlineStr">
         <is>
           <t>C.a k.
 C. a k.</t>
         </is>
       </c>
-      <c r="F4" s="18" t="inlineStr">
+      <c r="F4" s="16" t="inlineStr">
         <is>
           <t>C.&amp;nbsp;a&amp;nbsp;k.
 C.&amp;nbsp;a&amp;nbsp;k.</t>
@@ -587,12 +585,11 @@
           <t>2026-05-20T03:11:14.709599</t>
         </is>
       </c>
-      <c r="L4" s="11" t="n"/>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>C:\Users\ocape\IdeaProjects\TypofixAppTest\tests\resources\selenium-element-screenshot-11.png</t>
-        </is>
-      </c>
+      <c r="L4" s="11">
+        <f>HYPERLINK("C:\Users\ocape\IdeaProjects\TypofixAppTest\results\selenium-element-screenshot-11.png", "LINK")</f>
+        <v/>
+      </c>
+      <c r="M4" s="11" t="n"/>
     </row>
     <row r="5" ht="12.75" customHeight="1" s="12">
       <c r="A5" s="15" t="inlineStr">
@@ -607,13 +604,13 @@
           <t>Czech (traditional rules)</t>
         </is>
       </c>
-      <c r="E5" s="18" t="inlineStr">
+      <c r="E5" s="16" t="inlineStr">
         <is>
           <t>C.a k.
 C. a k.</t>
         </is>
       </c>
-      <c r="F5" s="18" t="inlineStr">
+      <c r="F5" s="16" t="inlineStr">
         <is>
           <t>C.&amp;nbsp;a&amp;nbsp;k.
 C.&amp;nbsp;a&amp;nbsp;k.</t>
@@ -637,12 +634,11 @@
           <t>2026-05-20T03:11:25.879240</t>
         </is>
       </c>
-      <c r="L5" s="11" t="n"/>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>C:\Users\ocape\IdeaProjects\TypofixAppTest\tests\resources\selenium-element-screenshot-12.png</t>
-        </is>
-      </c>
+      <c r="L5" s="11">
+        <f>HYPERLINK("C:\Users\ocape\IdeaProjects\TypofixAppTest\results\selenium-element-screenshot-12.png", "LINK")</f>
+        <v/>
+      </c>
+      <c r="M5" s="11" t="n"/>
     </row>
     <row r="6" ht="12.75" customHeight="1" s="12">
       <c r="A6" s="15" t="n"/>
@@ -9199,14 +9195,14 @@
           <t>English</t>
         </is>
       </c>
-      <c r="E2" s="18" t="inlineStr">
+      <c r="E2" s="16" t="inlineStr">
         <is>
           <t>rock‘n’roll
 rock' n' roll
 rock’n’roll</t>
         </is>
       </c>
-      <c r="F2" s="18" t="inlineStr">
+      <c r="F2" s="16" t="inlineStr">
         <is>
           <t>rock ’n’ roll
 rock ’n’ roll
@@ -9228,7 +9224,7 @@
           <t>English (UK)</t>
         </is>
       </c>
-      <c r="E3" s="18" t="inlineStr">
+      <c r="E3" s="16" t="inlineStr">
         <is>
           <t>rock‘n’roll
 rock' n' roll
@@ -9264,7 +9260,7 @@
 rock’n’roll</t>
         </is>
       </c>
-      <c r="F4" s="18" t="inlineStr">
+      <c r="F4" s="16" t="inlineStr">
         <is>
           <t>rock ’n’ roll
 rock ’n’ roll
@@ -9286,14 +9282,14 @@
           <t>German (Germany)</t>
         </is>
       </c>
-      <c r="E5" s="18" t="inlineStr">
+      <c r="E5" s="16" t="inlineStr">
         <is>
           <t>rock‘n’roll
 rock' n' roll
 rock’n’roll</t>
         </is>
       </c>
-      <c r="F5" s="18" t="inlineStr">
+      <c r="F5" s="16" t="inlineStr">
         <is>
           <t>rock ’n’ roll
 rock ’n’ roll
@@ -9315,14 +9311,14 @@
           <t>Spanish</t>
         </is>
       </c>
-      <c r="E6" s="18" t="inlineStr">
+      <c r="E6" s="16" t="inlineStr">
         <is>
           <t>rock‘n’roll
 rock' n' roll
 rock’n’roll</t>
         </is>
       </c>
-      <c r="F6" s="18" t="inlineStr">
+      <c r="F6" s="16" t="inlineStr">
         <is>
           <t>rock ’n’ roll
 rock ’n’ roll
@@ -9344,14 +9340,14 @@
           <t>Czech (academic rules)</t>
         </is>
       </c>
-      <c r="E7" s="18" t="inlineStr">
+      <c r="E7" s="16" t="inlineStr">
         <is>
           <t>Guns’N’Roses
 Guns n'Roses
 Guns ‘N’ Roses</t>
         </is>
       </c>
-      <c r="F7" s="18" t="inlineStr">
+      <c r="F7" s="16" t="inlineStr">
         <is>
           <t>Guns N’ Roses
 Guns N’ Roses
@@ -9373,14 +9369,14 @@
           <t>Czech (traditional rules)</t>
         </is>
       </c>
-      <c r="E8" s="15" t="inlineStr">
+      <c r="E8" s="16" t="inlineStr">
         <is>
           <t>Guns’N’Roses
 Guns n'Roses
 Guns ‘N’ Roses</t>
         </is>
       </c>
-      <c r="F8" s="18" t="inlineStr">
+      <c r="F8" s="16" t="inlineStr">
         <is>
           <t>Guns N’ Roses
 Guns N’ Roses
@@ -9402,14 +9398,14 @@
           <t>English</t>
         </is>
       </c>
-      <c r="E9" s="18" t="inlineStr">
+      <c r="E9" s="16" t="inlineStr">
         <is>
           <t>Guns’N’Roses
 Guns n'Roses
 Guns ‘N’ Roses</t>
         </is>
       </c>
-      <c r="F9" s="18" t="inlineStr">
+      <c r="F9" s="16" t="inlineStr">
         <is>
           <t>Guns N’ Roses
 Guns N’ Roses
@@ -9431,14 +9427,14 @@
           <t>English (UK)</t>
         </is>
       </c>
-      <c r="E10" s="18" t="inlineStr">
+      <c r="E10" s="16" t="inlineStr">
         <is>
           <t>Guns’N’Roses
 Guns n'Roses
 Guns ‘N’ Roses</t>
         </is>
       </c>
-      <c r="F10" s="18" t="inlineStr">
+      <c r="F10" s="16" t="inlineStr">
         <is>
           <t>Guns N’ Roses
 Guns N’ Roses
@@ -9460,14 +9456,14 @@
           <t>English (US)</t>
         </is>
       </c>
-      <c r="E11" s="18" t="inlineStr">
+      <c r="E11" s="16" t="inlineStr">
         <is>
           <t>Guns’N’Roses
 Guns n'Roses
 Guns ‘N’ Roses</t>
         </is>
       </c>
-      <c r="F11" s="18" t="inlineStr">
+      <c r="F11" s="16" t="inlineStr">
         <is>
           <t>Guns N’ Roses
 Guns N’ Roses
@@ -9489,14 +9485,14 @@
           <t>German (Germany)</t>
         </is>
       </c>
-      <c r="E12" s="15" t="inlineStr">
+      <c r="E12" s="16" t="inlineStr">
         <is>
           <t>Guns’N’Roses
 Guns n'Roses
 Guns ‘N’ Roses</t>
         </is>
       </c>
-      <c r="F12" s="18" t="inlineStr">
+      <c r="F12" s="16" t="inlineStr">
         <is>
           <t>Guns N’ Roses
 Guns N’ Roses
@@ -9518,14 +9514,14 @@
           <t>Spanish</t>
         </is>
       </c>
-      <c r="E13" s="18" t="inlineStr">
+      <c r="E13" s="16" t="inlineStr">
         <is>
           <t>Guns’N’Roses
 Guns n'Roses
 Guns ‘N’ Roses</t>
         </is>
       </c>
-      <c r="F13" s="15" t="inlineStr">
+      <c r="F13" s="16" t="inlineStr">
         <is>
           <t>Guns N’ Roses
 Guns N’ Roses
@@ -9547,13 +9543,13 @@
           <t>Czech (academic rules)</t>
         </is>
       </c>
-      <c r="E14" s="18" t="inlineStr">
+      <c r="E14" s="16" t="inlineStr">
         <is>
           <t>C.a k.
 C. a k.</t>
         </is>
       </c>
-      <c r="F14" s="15" t="inlineStr">
+      <c r="F14" s="16" t="inlineStr">
         <is>
           <t>C.&amp;nbsp;a&amp;nbsp;k.
 C.&amp;nbsp;a&amp;nbsp;k.</t>
@@ -9574,13 +9570,13 @@
           <t>Czech (traditional rules)</t>
         </is>
       </c>
-      <c r="E15" s="18" t="inlineStr">
+      <c r="E15" s="16" t="inlineStr">
         <is>
           <t>C.a k.
 C. a k.</t>
         </is>
       </c>
-      <c r="F15" s="18" t="inlineStr">
+      <c r="F15" s="16" t="inlineStr">
         <is>
           <t>C.&amp;nbsp;a&amp;nbsp;k.
 C.&amp;nbsp;a&amp;nbsp;k.</t>
@@ -9601,14 +9597,14 @@
           <t>Italian</t>
         </is>
       </c>
-      <c r="E16" s="15" t="inlineStr">
+      <c r="E16" s="16" t="inlineStr">
         <is>
           <t>E' (Italian)
 E’ (Italian)
 E` (Italian)</t>
         </is>
       </c>
-      <c r="F16" s="15" t="inlineStr">
+      <c r="F16" s="16" t="inlineStr">
         <is>
           <t>È (Italian)
 È (Italian)
@@ -9863,7 +9859,7 @@
 lij́n (Dutch)</t>
         </is>
       </c>
-      <c r="F28" s="18" t="inlineStr">
+      <c r="F28" s="16" t="inlineStr">
         <is>
           <t>líȷ́n (Dutch)
 líȷ́n (Dutch)</t>
@@ -10009,14 +10005,14 @@
           <t>Czech (academic rules)</t>
         </is>
       </c>
-      <c r="E34" s="18" t="inlineStr">
+      <c r="E34" s="16" t="inlineStr">
         <is>
           <t>Author et all
 Author et al
 Author et all.</t>
         </is>
       </c>
-      <c r="F34" s="18" t="inlineStr">
+      <c r="F34" s="16" t="inlineStr">
         <is>
           <t>Author et&amp;nbsp;al.
 Author et&amp;nbsp;al.
@@ -10038,14 +10034,14 @@
           <t>Czech (traditional rules)</t>
         </is>
       </c>
-      <c r="E35" s="18" t="inlineStr">
+      <c r="E35" s="16" t="inlineStr">
         <is>
           <t>Author et all
 Author et al
 Author et all.</t>
         </is>
       </c>
-      <c r="F35" s="18" t="inlineStr">
+      <c r="F35" s="16" t="inlineStr">
         <is>
           <t>Author et&amp;nbsp;al.
 Author et&amp;nbsp;al.
@@ -10067,14 +10063,14 @@
           <t>English (UK)</t>
         </is>
       </c>
-      <c r="E36" s="18" t="inlineStr">
+      <c r="E36" s="16" t="inlineStr">
         <is>
           <t>Author et all
 Author et al
 Author et all.</t>
         </is>
       </c>
-      <c r="F36" s="18" t="inlineStr">
+      <c r="F36" s="16" t="inlineStr">
         <is>
           <t>Author et&amp;nbsp;al.
 Author et&amp;nbsp;al.
@@ -10096,14 +10092,14 @@
           <t>English (US)</t>
         </is>
       </c>
-      <c r="E37" s="15" t="inlineStr">
+      <c r="E37" s="16" t="inlineStr">
         <is>
           <t>Author et all
 Author et al
 Author et all.</t>
         </is>
       </c>
-      <c r="F37" s="18" t="inlineStr">
+      <c r="F37" s="16" t="inlineStr">
         <is>
           <t>Author et&amp;nbsp;al.
 Author et&amp;nbsp;al.
@@ -18999,7 +18995,7 @@
           <t>English</t>
         </is>
       </c>
-      <c r="E2" s="18" t="inlineStr">
+      <c r="E2" s="16" t="inlineStr">
         <is>
           <t>rock‘n’roll
 rock' n' roll
@@ -19028,14 +19024,14 @@
           <t>English (UK)</t>
         </is>
       </c>
-      <c r="E3" s="18" t="inlineStr">
+      <c r="E3" s="16" t="inlineStr">
         <is>
           <t>rock‘n’roll
 rock' n' roll
 rock’n’roll</t>
         </is>
       </c>
-      <c r="F3" s="18" t="inlineStr">
+      <c r="F3" s="16" t="inlineStr">
         <is>
           <t>rock ’n’ roll
 rock ’n’ roll
@@ -19057,14 +19053,14 @@
           <t>English (US)</t>
         </is>
       </c>
-      <c r="E4" s="15" t="inlineStr">
+      <c r="E4" s="16" t="inlineStr">
         <is>
           <t>rock‘n’roll
 rock' n' roll
 rock’n’roll</t>
         </is>
       </c>
-      <c r="F4" s="18" t="inlineStr">
+      <c r="F4" s="16" t="inlineStr">
         <is>
           <t>rock ’n’ roll
 rock ’n’ roll
@@ -19086,7 +19082,7 @@
           <t>German (Germany)</t>
         </is>
       </c>
-      <c r="E5" s="18" t="inlineStr">
+      <c r="E5" s="16" t="inlineStr">
         <is>
           <t>rock‘n’roll
 rock' n' roll
@@ -19115,7 +19111,7 @@
           <t>Spanish</t>
         </is>
       </c>
-      <c r="E6" s="18" t="inlineStr">
+      <c r="E6" s="16" t="inlineStr">
         <is>
           <t>rock‘n’roll
 rock' n' roll
@@ -19144,14 +19140,14 @@
           <t>Czech (academic rules)</t>
         </is>
       </c>
-      <c r="E7" s="18" t="inlineStr">
+      <c r="E7" s="16" t="inlineStr">
         <is>
           <t>Guns’N’Roses
 Guns n'Roses
 Guns ‘N’ Roses</t>
         </is>
       </c>
-      <c r="F7" s="18" t="inlineStr">
+      <c r="F7" s="16" t="inlineStr">
         <is>
           <t>Guns N’ Roses
 Guns N’ Roses
@@ -19173,14 +19169,14 @@
           <t>Czech (traditional rules)</t>
         </is>
       </c>
-      <c r="E8" s="18" t="inlineStr">
+      <c r="E8" s="16" t="inlineStr">
         <is>
           <t>Guns’N’Roses
 Guns n'Roses
 Guns ‘N’ Roses</t>
         </is>
       </c>
-      <c r="F8" s="18" t="inlineStr">
+      <c r="F8" s="16" t="inlineStr">
         <is>
           <t>Guns N’ Roses
 Guns N’ Roses
@@ -19202,7 +19198,7 @@
           <t>English</t>
         </is>
       </c>
-      <c r="E9" s="18" t="inlineStr">
+      <c r="E9" s="16" t="inlineStr">
         <is>
           <t>Guns’N’Roses
 Guns n'Roses
@@ -19231,14 +19227,14 @@
           <t>English (UK)</t>
         </is>
       </c>
-      <c r="E10" s="18" t="inlineStr">
+      <c r="E10" s="16" t="inlineStr">
         <is>
           <t>Guns’N’Roses
 Guns n'Roses
 Guns ‘N’ Roses</t>
         </is>
       </c>
-      <c r="F10" s="18" t="inlineStr">
+      <c r="F10" s="16" t="inlineStr">
         <is>
           <t>Guns N’ Roses
 Guns N’ Roses
@@ -19260,14 +19256,14 @@
           <t>English (US)</t>
         </is>
       </c>
-      <c r="E11" s="18" t="inlineStr">
+      <c r="E11" s="16" t="inlineStr">
         <is>
           <t>Guns’N’Roses
 Guns n'Roses
 Guns ‘N’ Roses</t>
         </is>
       </c>
-      <c r="F11" s="18" t="inlineStr">
+      <c r="F11" s="16" t="inlineStr">
         <is>
           <t>Guns N’ Roses
 Guns N’ Roses
@@ -19289,14 +19285,14 @@
           <t>German (Germany)</t>
         </is>
       </c>
-      <c r="E12" s="18" t="inlineStr">
+      <c r="E12" s="16" t="inlineStr">
         <is>
           <t>Guns’N’Roses
 Guns n'Roses
 Guns ‘N’ Roses</t>
         </is>
       </c>
-      <c r="F12" s="18" t="inlineStr">
+      <c r="F12" s="16" t="inlineStr">
         <is>
           <t>Guns N’ Roses
 Guns N’ Roses
@@ -19318,14 +19314,14 @@
           <t>Spanish</t>
         </is>
       </c>
-      <c r="E13" s="18" t="inlineStr">
+      <c r="E13" s="16" t="inlineStr">
         <is>
           <t>Guns’N’Roses
 Guns n'Roses
 Guns ‘N’ Roses</t>
         </is>
       </c>
-      <c r="F13" s="18" t="inlineStr">
+      <c r="F13" s="16" t="inlineStr">
         <is>
           <t>Guns N’ Roses
 Guns N’ Roses
@@ -19347,13 +19343,13 @@
           <t>Czech (academic rules)</t>
         </is>
       </c>
-      <c r="E14" s="18" t="inlineStr">
+      <c r="E14" s="16" t="inlineStr">
         <is>
           <t>C.a k.
 C. a k.</t>
         </is>
       </c>
-      <c r="F14" s="18" t="inlineStr">
+      <c r="F14" s="16" t="inlineStr">
         <is>
           <t>C.&amp;nbsp;a&amp;nbsp;k.
 C.&amp;nbsp;a&amp;nbsp;k.</t>
@@ -19374,13 +19370,13 @@
           <t>Czech (traditional rules)</t>
         </is>
       </c>
-      <c r="E15" s="18" t="inlineStr">
+      <c r="E15" s="16" t="inlineStr">
         <is>
           <t>C.a k.
 C. a k.</t>
         </is>
       </c>
-      <c r="F15" s="18" t="inlineStr">
+      <c r="F15" s="16" t="inlineStr">
         <is>
           <t>C.&amp;nbsp;a&amp;nbsp;k.
 C.&amp;nbsp;a&amp;nbsp;k.</t>
@@ -19401,14 +19397,14 @@
           <t>Italian</t>
         </is>
       </c>
-      <c r="E16" s="18" t="inlineStr">
+      <c r="E16" s="16" t="inlineStr">
         <is>
           <t>E' (Italian)
 E’ (Italian)
 E` (Italian)</t>
         </is>
       </c>
-      <c r="F16" s="18" t="inlineStr">
+      <c r="F16" s="16" t="inlineStr">
         <is>
           <t>È (Italian)
 È (Italian)
@@ -19657,13 +19653,13 @@
           <t>Dutch</t>
         </is>
       </c>
-      <c r="E28" s="18" t="inlineStr">
+      <c r="E28" s="16" t="inlineStr">
         <is>
           <t>liȷ́n (Dutch)
 lij́n (Dutch)</t>
         </is>
       </c>
-      <c r="F28" s="18" t="inlineStr">
+      <c r="F28" s="16" t="inlineStr">
         <is>
           <t>líȷ́n (Dutch)
 líȷ́n (Dutch)</t>
@@ -19809,14 +19805,14 @@
           <t>Czech (academic rules)</t>
         </is>
       </c>
-      <c r="E34" s="18" t="inlineStr">
+      <c r="E34" s="16" t="inlineStr">
         <is>
           <t>Author et all
 Author et al
 Author et all.</t>
         </is>
       </c>
-      <c r="F34" s="18" t="inlineStr">
+      <c r="F34" s="16" t="inlineStr">
         <is>
           <t>Author et&amp;nbsp;al.
 Author et&amp;nbsp;al.
@@ -19838,14 +19834,14 @@
           <t>Czech (traditional rules)</t>
         </is>
       </c>
-      <c r="E35" s="18" t="inlineStr">
+      <c r="E35" s="16" t="inlineStr">
         <is>
           <t>Author et all
 Author et al
 Author et all.</t>
         </is>
       </c>
-      <c r="F35" s="18" t="inlineStr">
+      <c r="F35" s="16" t="inlineStr">
         <is>
           <t>Author et&amp;nbsp;al.
 Author et&amp;nbsp;al.
@@ -19867,14 +19863,14 @@
           <t>English (UK)</t>
         </is>
       </c>
-      <c r="E36" s="18" t="inlineStr">
+      <c r="E36" s="16" t="inlineStr">
         <is>
           <t>Author et all
 Author et al
 Author et all.</t>
         </is>
       </c>
-      <c r="F36" s="18" t="inlineStr">
+      <c r="F36" s="16" t="inlineStr">
         <is>
           <t>Author et&amp;nbsp;al.
 Author et&amp;nbsp;al.
@@ -19896,14 +19892,14 @@
           <t>English (US)</t>
         </is>
       </c>
-      <c r="E37" s="18" t="inlineStr">
+      <c r="E37" s="16" t="inlineStr">
         <is>
           <t>Author et all
 Author et al
 Author et all.</t>
         </is>
       </c>
-      <c r="F37" s="18" t="inlineStr">
+      <c r="F37" s="16" t="inlineStr">
         <is>
           <t>Author et&amp;nbsp;al.
 Author et&amp;nbsp;al.
@@ -28791,13 +28787,13 @@
           <t>Czech (academic rules)</t>
         </is>
       </c>
-      <c r="E2" s="18" t="inlineStr">
+      <c r="E2" s="16" t="inlineStr">
         <is>
           <t>C.a k.
 C. a k.</t>
         </is>
       </c>
-      <c r="F2" s="18" t="inlineStr">
+      <c r="F2" s="16" t="inlineStr">
         <is>
           <t>C.&amp;nbsp;a&amp;nbsp;k.
 C.&amp;nbsp;a&amp;nbsp;k.</t>

</xml_diff>